<commit_message>
fix: DSCALE convergence beta, electricity GWh→TJ, and 6 edge case bugs
- DSCALE convergence now uses per-country ENSHORT beta (matching official
  Energy_demand_downs_1.py:661), falls back to regional ENLONG beta
- GCAM+IEA electricity converted from GWh to TJ (×3.6) via new
  iea_unit_factor; fixes electrification_rate cross-unit mismatch
- Population guard in ENSHORT reduced from 1.0M to 1e-6 (~1 person)
- DSCALE non-TFC outputs now properly written to disk (was early-returning
  in run_indicator before write_output_for)
- LogLogFunc degenerate beta=0 -> None fixed to beta=1.0
- Zero-IEA-sum regions now use equal split instead of leaking to global
  residual
- IO defensive warnings for missing Units column and missing filter_col
- +58 tests: 24 cross-validation against official DSCALE, 34 edge cases
- +36 conservation sum-equality tests (was only NaN check)
- 231/231 tests pass, 96/96 pipeline OK

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/compare/output/dscale_TFC_downscaled_SSP126.xlsx
+++ b/compare/output/dscale_TFC_downscaled_SSP126.xlsx
@@ -4478,58 +4478,58 @@
         </is>
       </c>
       <c r="E54" t="n">
-        <v>2113369.234199</v>
+        <v>4023598.886803</v>
       </c>
       <c r="F54" t="n">
-        <v>2676218.855651</v>
+        <v>5090337.966967</v>
       </c>
       <c r="G54" t="n">
-        <v>2854651.963151</v>
+        <v>5403985.383615</v>
       </c>
       <c r="H54" t="n">
-        <v>2981010.450494</v>
+        <v>5605437.008039</v>
       </c>
       <c r="I54" t="n">
-        <v>3130898.124877</v>
+        <v>5841059.070572</v>
       </c>
       <c r="J54" t="n">
-        <v>3289249.775077</v>
+        <v>6082224.42599</v>
       </c>
       <c r="K54" t="n">
-        <v>3739127.160903</v>
+        <v>6336984.302821</v>
       </c>
       <c r="L54" t="n">
-        <v>4177468.601591</v>
+        <v>6596513.570113</v>
       </c>
       <c r="M54" t="n">
-        <v>4599839.197186</v>
+        <v>6851732.732094</v>
       </c>
       <c r="N54" t="n">
-        <v>4989083.536158</v>
+        <v>7077724.641003</v>
       </c>
       <c r="O54" t="n">
-        <v>5321210.867297</v>
+        <v>7249126.035091</v>
       </c>
       <c r="P54" t="n">
-        <v>5606078.629823</v>
+        <v>7380751.384625</v>
       </c>
       <c r="Q54" t="n">
-        <v>5839313.614715</v>
+        <v>7463613.770868</v>
       </c>
       <c r="R54" t="n">
-        <v>6005057.452614</v>
+        <v>7482913.730104</v>
       </c>
       <c r="S54" t="n">
-        <v>6102086.678211</v>
+        <v>7435196.687246</v>
       </c>
       <c r="T54" t="n">
-        <v>6136291.630273</v>
+        <v>7328484.947606</v>
       </c>
       <c r="U54" t="n">
-        <v>6119742.048108</v>
+        <v>7178662.972141</v>
       </c>
       <c r="V54" t="n">
-        <v>6065730.578093</v>
+        <v>7001689.802546</v>
       </c>
     </row>
     <row r="55">
@@ -4554,58 +4554,58 @@
         </is>
       </c>
       <c r="E55" t="n">
-        <v>2609406.800601</v>
+        <v>699177.147997</v>
       </c>
       <c r="F55" t="n">
-        <v>3245516.273929</v>
+        <v>831397.162613</v>
       </c>
       <c r="G55" t="n">
-        <v>3393954.705535</v>
+        <v>844621.285071</v>
       </c>
       <c r="H55" t="n">
-        <v>3475222.05247</v>
+        <v>850795.494924</v>
       </c>
       <c r="I55" t="n">
-        <v>3579788.341704</v>
+        <v>869627.396009</v>
       </c>
       <c r="J55" t="n">
-        <v>3687264.032447</v>
+        <v>894289.381534</v>
       </c>
       <c r="K55" t="n">
-        <v>3522270.684764</v>
+        <v>924413.5428460001</v>
       </c>
       <c r="L55" t="n">
-        <v>3376628.10991</v>
+        <v>957583.141388</v>
       </c>
       <c r="M55" t="n">
-        <v>3243560.612347</v>
+        <v>991667.077439</v>
       </c>
       <c r="N55" t="n">
-        <v>3111627.820186</v>
+        <v>1022986.715342</v>
       </c>
       <c r="O55" t="n">
-        <v>2977403.620572</v>
+        <v>1049488.452778</v>
       </c>
       <c r="P55" t="n">
-        <v>2848670.34707</v>
+        <v>1073997.592268</v>
       </c>
       <c r="Q55" t="n">
-        <v>2718852.794939</v>
+        <v>1094552.638786</v>
       </c>
       <c r="R55" t="n">
-        <v>2587823.618398</v>
+        <v>1109967.340908</v>
       </c>
       <c r="S55" t="n">
-        <v>2451212.578284</v>
+        <v>1118102.56925</v>
       </c>
       <c r="T55" t="n">
-        <v>2310885.031052</v>
+        <v>1118691.713718</v>
       </c>
       <c r="U55" t="n">
-        <v>2171265.082813</v>
+        <v>1112344.15878</v>
       </c>
       <c r="V55" t="n">
-        <v>2036774.121218</v>
+        <v>1100814.896765</v>
       </c>
     </row>
     <row r="56">
@@ -6910,58 +6910,58 @@
         </is>
       </c>
       <c r="E86" t="n">
-        <v>905532.597388</v>
+        <v>467324.559837</v>
       </c>
       <c r="F86" t="n">
-        <v>991760.879097</v>
+        <v>503843.65611</v>
       </c>
       <c r="G86" t="n">
-        <v>1030248.255548</v>
+        <v>520170.654857</v>
       </c>
       <c r="H86" t="n">
-        <v>1032196.427617</v>
+        <v>523898.722448</v>
       </c>
       <c r="I86" t="n">
-        <v>1030116.191904</v>
+        <v>529151.354407</v>
       </c>
       <c r="J86" t="n">
-        <v>1016192.276823</v>
+        <v>528974.768509</v>
       </c>
       <c r="K86" t="n">
-        <v>995551.945663</v>
+        <v>524070.607958</v>
       </c>
       <c r="L86" t="n">
-        <v>970359.8370159999</v>
+        <v>515444.874821</v>
       </c>
       <c r="M86" t="n">
-        <v>940251.600527</v>
+        <v>503465.346785</v>
       </c>
       <c r="N86" t="n">
-        <v>902558.225353</v>
+        <v>486854.130829</v>
       </c>
       <c r="O86" t="n">
-        <v>857745.0211219999</v>
+        <v>465735.928963</v>
       </c>
       <c r="P86" t="n">
-        <v>811972.150177</v>
+        <v>443543.848491</v>
       </c>
       <c r="Q86" t="n">
-        <v>767903.603348</v>
+        <v>421803.09531</v>
       </c>
       <c r="R86" t="n">
-        <v>724870.333279</v>
+        <v>400469.056218</v>
       </c>
       <c r="S86" t="n">
-        <v>683757.374468</v>
+        <v>380143.189633</v>
       </c>
       <c r="T86" t="n">
-        <v>642161.641087</v>
+        <v>359379.465715</v>
       </c>
       <c r="U86" t="n">
-        <v>599791.056676</v>
+        <v>337570.65789</v>
       </c>
       <c r="V86" t="n">
-        <v>557976.872774</v>
+        <v>315433.694923</v>
       </c>
     </row>
     <row r="87">
@@ -6986,58 +6986,58 @@
         </is>
       </c>
       <c r="E87" t="n">
-        <v>132270.792138</v>
+        <v>68261.91557700001</v>
       </c>
       <c r="F87" t="n">
-        <v>162345.677844</v>
+        <v>82476.37268499999</v>
       </c>
       <c r="G87" t="n">
-        <v>190941.273843</v>
+        <v>96405.93606399999</v>
       </c>
       <c r="H87" t="n">
-        <v>210880.3226</v>
+        <v>107033.824807</v>
       </c>
       <c r="I87" t="n">
-        <v>227047.556678</v>
+        <v>116630.068603</v>
       </c>
       <c r="J87" t="n">
-        <v>238435.685443</v>
+        <v>124116.729076</v>
       </c>
       <c r="K87" t="n">
-        <v>246527.119971</v>
+        <v>129774.863285</v>
       </c>
       <c r="L87" t="n">
-        <v>252269.210911</v>
+        <v>134002.734737</v>
       </c>
       <c r="M87" t="n">
-        <v>255848.567643</v>
+        <v>136996.190978</v>
       </c>
       <c r="N87" t="n">
-        <v>256645.681351</v>
+        <v>138438.725187</v>
       </c>
       <c r="O87" t="n">
-        <v>253656.228077</v>
+        <v>137729.530468</v>
       </c>
       <c r="P87" t="n">
-        <v>247590.651587</v>
+        <v>135247.631869</v>
       </c>
       <c r="Q87" t="n">
-        <v>238646.23003</v>
+        <v>131086.39948</v>
       </c>
       <c r="R87" t="n">
-        <v>226958.492003</v>
+        <v>125387.74029</v>
       </c>
       <c r="S87" t="n">
-        <v>213389.449572</v>
+        <v>118636.447698</v>
       </c>
       <c r="T87" t="n">
-        <v>197879.283189</v>
+        <v>110741.20053</v>
       </c>
       <c r="U87" t="n">
-        <v>181720.837896</v>
+        <v>102274.987461</v>
       </c>
       <c r="V87" t="n">
-        <v>166078.709754</v>
+        <v>93887.08317899999</v>
       </c>
     </row>
     <row r="88">
@@ -7062,58 +7062,58 @@
         </is>
       </c>
       <c r="E88" t="n">
-        <v>2298929.239014</v>
+        <v>1186424.539346</v>
       </c>
       <c r="F88" t="n">
-        <v>2250176.613901</v>
+        <v>1143155.810979</v>
       </c>
       <c r="G88" t="n">
-        <v>2152597.237626</v>
+        <v>1086842.815516</v>
       </c>
       <c r="H88" t="n">
-        <v>2091585.358684</v>
+        <v>1061599.195644</v>
       </c>
       <c r="I88" t="n">
-        <v>2100258.724834</v>
+        <v>1078863.488978</v>
       </c>
       <c r="J88" t="n">
-        <v>2129485.546545</v>
+        <v>1108495.065076</v>
       </c>
       <c r="K88" t="n">
-        <v>2162619.350183</v>
+        <v>1138429.031825</v>
       </c>
       <c r="L88" t="n">
-        <v>2192308.53307</v>
+        <v>1164531.088665</v>
       </c>
       <c r="M88" t="n">
-        <v>2218053.993685</v>
+        <v>1187675.003681</v>
       </c>
       <c r="N88" t="n">
-        <v>2237319.502687</v>
+        <v>1206845.399299</v>
       </c>
       <c r="O88" t="n">
-        <v>2241231.245765</v>
+        <v>1216937.307201</v>
       </c>
       <c r="P88" t="n">
-        <v>2231448.931465</v>
+        <v>1218940.140443</v>
       </c>
       <c r="Q88" t="n">
-        <v>2206844.24537</v>
+        <v>1212201.283476</v>
       </c>
       <c r="R88" t="n">
-        <v>2164868.302912</v>
+        <v>1196024.621646</v>
       </c>
       <c r="S88" t="n">
-        <v>2110878.878703</v>
+        <v>1173568.666083</v>
       </c>
       <c r="T88" t="n">
-        <v>2052199.144682</v>
+        <v>1148493.128472</v>
       </c>
       <c r="U88" t="n">
-        <v>1994948.874621</v>
+        <v>1122784.670707</v>
       </c>
       <c r="V88" t="n">
-        <v>1941120.896449</v>
+        <v>1097348.23527</v>
       </c>
     </row>
     <row r="89">
@@ -7138,58 +7138,58 @@
         </is>
       </c>
       <c r="E89" t="n">
-        <v>257963.622751</v>
+        <v>133129.096405</v>
       </c>
       <c r="F89" t="n">
-        <v>267899.790515</v>
+        <v>136100.962207</v>
       </c>
       <c r="G89" t="n">
-        <v>276386.249193</v>
+        <v>139546.964008</v>
       </c>
       <c r="H89" t="n">
-        <v>277223.541619</v>
+        <v>140706.802892</v>
       </c>
       <c r="I89" t="n">
-        <v>277716.291202</v>
+        <v>142657.64657</v>
       </c>
       <c r="J89" t="n">
-        <v>274900.178839</v>
+        <v>143098.173231</v>
       </c>
       <c r="K89" t="n">
-        <v>270458.551742</v>
+        <v>142372.658962</v>
       </c>
       <c r="L89" t="n">
-        <v>266114.893901</v>
+        <v>141357.414994</v>
       </c>
       <c r="M89" t="n">
-        <v>263228.883209</v>
+        <v>140948.040816</v>
       </c>
       <c r="N89" t="n">
-        <v>261407.595194</v>
+        <v>141007.37656</v>
       </c>
       <c r="O89" t="n">
-        <v>259377.992628</v>
+        <v>140836.317757</v>
       </c>
       <c r="P89" t="n">
-        <v>257088.020906</v>
+        <v>140435.617365</v>
       </c>
       <c r="Q89" t="n">
-        <v>254573.09838</v>
+        <v>139834.896478</v>
       </c>
       <c r="R89" t="n">
-        <v>251500.250744</v>
+        <v>138946.323818</v>
       </c>
       <c r="S89" t="n">
-        <v>248140.610593</v>
+        <v>137956.776352</v>
       </c>
       <c r="T89" t="n">
-        <v>244026.251171</v>
+        <v>136566.898667</v>
       </c>
       <c r="U89" t="n">
-        <v>239397.095051</v>
+        <v>134735.978428</v>
       </c>
       <c r="V89" t="n">
-        <v>235140.771353</v>
+        <v>132929.026191</v>
       </c>
     </row>
     <row r="90">
@@ -7214,58 +7214,58 @@
         </is>
       </c>
       <c r="E90" t="n">
-        <v>28247.467411</v>
+        <v>883215.484635</v>
       </c>
       <c r="F90" t="n">
-        <v>53966.535994</v>
+        <v>919438.505337</v>
       </c>
       <c r="G90" t="n">
-        <v>76542.424246</v>
+        <v>963561.1938069999</v>
       </c>
       <c r="H90" t="n">
-        <v>96010.742167</v>
+        <v>996060.050531</v>
       </c>
       <c r="I90" t="n">
-        <v>114611.604454</v>
+        <v>1030440.373551</v>
       </c>
       <c r="J90" t="n">
-        <v>131298.076749</v>
+        <v>1047990.539466</v>
       </c>
       <c r="K90" t="n">
-        <v>146336.425036</v>
+        <v>1054442.239571</v>
       </c>
       <c r="L90" t="n">
-        <v>160079.49698</v>
+        <v>1055544.772674</v>
       </c>
       <c r="M90" t="n">
-        <v>172423.221802</v>
+        <v>1055256.865257</v>
       </c>
       <c r="N90" t="n">
-        <v>182720.580835</v>
+        <v>1050300.930153</v>
       </c>
       <c r="O90" t="n">
-        <v>190127.763891</v>
+        <v>1036466.076927</v>
       </c>
       <c r="P90" t="n">
-        <v>195180.759738</v>
+        <v>1015986.632172</v>
       </c>
       <c r="Q90" t="n">
-        <v>198561.766213</v>
+        <v>991106.445854</v>
       </c>
       <c r="R90" t="n">
-        <v>200609.657843</v>
+        <v>962904.465978</v>
       </c>
       <c r="S90" t="n">
-        <v>201904.316531</v>
+        <v>934137.746058</v>
       </c>
       <c r="T90" t="n">
-        <v>201887.006522</v>
+        <v>903815.396391</v>
       </c>
       <c r="U90" t="n">
-        <v>201126.578134</v>
+        <v>872165.931334</v>
       </c>
       <c r="V90" t="n">
-        <v>200216.449914</v>
+        <v>840900.796324</v>
       </c>
     </row>
     <row r="91">
@@ -7290,58 +7290,58 @@
         </is>
       </c>
       <c r="E91" t="n">
-        <v>534611.6959779999</v>
+        <v>275900.80824</v>
       </c>
       <c r="F91" t="n">
-        <v>580655.428287</v>
+        <v>294990.012305</v>
       </c>
       <c r="G91" t="n">
-        <v>602588.514116</v>
+        <v>304245.952671</v>
       </c>
       <c r="H91" t="n">
-        <v>592368.066565</v>
+        <v>300660.673675</v>
       </c>
       <c r="I91" t="n">
-        <v>571628.444338</v>
+        <v>293634.803449</v>
       </c>
       <c r="J91" t="n">
-        <v>540943.336962</v>
+        <v>281585.860247</v>
       </c>
       <c r="K91" t="n">
-        <v>508184.018277</v>
+        <v>267514.225223</v>
       </c>
       <c r="L91" t="n">
-        <v>477530.602579</v>
+        <v>253659.201752</v>
       </c>
       <c r="M91" t="n">
-        <v>450887.265468</v>
+        <v>241431.243874</v>
       </c>
       <c r="N91" t="n">
-        <v>427450.133865</v>
+        <v>230573.338705</v>
       </c>
       <c r="O91" t="n">
-        <v>405406.925074</v>
+        <v>220126.688244</v>
       </c>
       <c r="P91" t="n">
-        <v>384538.648242</v>
+        <v>210056.160051</v>
       </c>
       <c r="Q91" t="n">
-        <v>364451.526256</v>
+        <v>200190.207723</v>
       </c>
       <c r="R91" t="n">
-        <v>344426.029613</v>
+        <v>190285.021587</v>
       </c>
       <c r="S91" t="n">
-        <v>324773.851289</v>
+        <v>180561.954208</v>
       </c>
       <c r="T91" t="n">
-        <v>304730.646754</v>
+        <v>170539.518418</v>
       </c>
       <c r="U91" t="n">
-        <v>285016.084214</v>
+        <v>160410.973099</v>
       </c>
       <c r="V91" t="n">
-        <v>267051.493895</v>
+        <v>150968.693443</v>
       </c>
     </row>
     <row r="92">
@@ -7366,58 +7366,58 @@
         </is>
       </c>
       <c r="E92" t="n">
-        <v>344515.735354</v>
+        <v>177796.652319</v>
       </c>
       <c r="F92" t="n">
-        <v>377633.735711</v>
+        <v>191849.02942</v>
       </c>
       <c r="G92" t="n">
-        <v>405229.466108</v>
+        <v>204599.692955</v>
       </c>
       <c r="H92" t="n">
-        <v>410102.746576</v>
+        <v>208150.5993</v>
       </c>
       <c r="I92" t="n">
-        <v>405320.886107</v>
+        <v>208205.73207</v>
       </c>
       <c r="J92" t="n">
-        <v>391464.466224</v>
+        <v>203775.2403</v>
       </c>
       <c r="K92" t="n">
-        <v>374055.229359</v>
+        <v>196907.205409</v>
       </c>
       <c r="L92" t="n">
-        <v>356170.912262</v>
+        <v>189194.218766</v>
       </c>
       <c r="M92" t="n">
-        <v>340553.609056</v>
+        <v>182352.192526</v>
       </c>
       <c r="N92" t="n">
-        <v>326336.090591</v>
+        <v>176030.830233</v>
       </c>
       <c r="O92" t="n">
-        <v>311744.117259</v>
+        <v>169269.925765</v>
       </c>
       <c r="P92" t="n">
-        <v>296835.174108</v>
+        <v>162147.698616</v>
       </c>
       <c r="Q92" t="n">
-        <v>281777.144293</v>
+        <v>154777.853799</v>
       </c>
       <c r="R92" t="n">
-        <v>266148.11812</v>
+        <v>147038.829959</v>
       </c>
       <c r="S92" t="n">
-        <v>250388.044346</v>
+        <v>139206.264353</v>
       </c>
       <c r="T92" t="n">
-        <v>233846.58485</v>
+        <v>130869.948228</v>
       </c>
       <c r="U92" t="n">
-        <v>217038.233943</v>
+        <v>122152.10381</v>
       </c>
       <c r="V92" t="n">
-        <v>201410.008656</v>
+        <v>113860.45968</v>
       </c>
     </row>
     <row r="93">
@@ -7442,58 +7442,58 @@
         </is>
       </c>
       <c r="E93" t="n">
-        <v>43197.100389</v>
+        <v>22293.030625</v>
       </c>
       <c r="F93" t="n">
-        <v>50009.422901</v>
+        <v>25406.255686</v>
       </c>
       <c r="G93" t="n">
-        <v>56720.118218</v>
+        <v>28637.89468</v>
       </c>
       <c r="H93" t="n">
-        <v>62019.63481</v>
+        <v>31478.511816</v>
       </c>
       <c r="I93" t="n">
-        <v>66695.450427</v>
+        <v>34260.201134</v>
       </c>
       <c r="J93" t="n">
-        <v>69657.48368200001</v>
+        <v>36259.920633</v>
       </c>
       <c r="K93" t="n">
-        <v>71044.10494200001</v>
+        <v>37398.47773</v>
       </c>
       <c r="L93" t="n">
-        <v>71210.702112</v>
+        <v>37826.371245</v>
       </c>
       <c r="M93" t="n">
-        <v>70372.367178</v>
+        <v>37681.454863</v>
       </c>
       <c r="N93" t="n">
-        <v>68627.012928</v>
+        <v>37018.492317</v>
       </c>
       <c r="O93" t="n">
-        <v>66036.816617</v>
+        <v>35856.481093</v>
       </c>
       <c r="P93" t="n">
-        <v>62998.468775</v>
+        <v>34413.228684</v>
       </c>
       <c r="Q93" t="n">
-        <v>59626.232506</v>
+        <v>32752.196139</v>
       </c>
       <c r="R93" t="n">
-        <v>55844.79381</v>
+        <v>30852.568859</v>
       </c>
       <c r="S93" t="n">
-        <v>51794.597104</v>
+        <v>28795.833265</v>
       </c>
       <c r="T93" t="n">
-        <v>47503.241268</v>
+        <v>26584.723182</v>
       </c>
       <c r="U93" t="n">
-        <v>43212.07187</v>
+        <v>24320.348508</v>
       </c>
       <c r="V93" t="n">
-        <v>39211.912178</v>
+        <v>22167.152344</v>
       </c>
     </row>
     <row r="94">
@@ -7518,58 +7518,58 @@
         </is>
       </c>
       <c r="E94" t="n">
-        <v>111175.7366</v>
+        <v>3119969.719884</v>
       </c>
       <c r="F94" t="n">
-        <v>216405.656574</v>
+        <v>3544370.316906</v>
       </c>
       <c r="G94" t="n">
-        <v>309228.171838</v>
+        <v>3767233.935218</v>
       </c>
       <c r="H94" t="n">
-        <v>388046.664778</v>
+        <v>3831225.75775</v>
       </c>
       <c r="I94" t="n">
-        <v>461425.93983</v>
+        <v>3864276.397622</v>
       </c>
       <c r="J94" t="n">
-        <v>526033.299316</v>
+        <v>3852271.821103</v>
       </c>
       <c r="K94" t="n">
-        <v>583616.5134310001</v>
+        <v>3820144.13725</v>
       </c>
       <c r="L94" t="n">
-        <v>635723.918401</v>
+        <v>3777008.491434</v>
       </c>
       <c r="M94" t="n">
-        <v>681431.635654</v>
+        <v>3724388.211019</v>
       </c>
       <c r="N94" t="n">
-        <v>718186.085309</v>
+        <v>3656700.815326</v>
       </c>
       <c r="O94" t="n">
-        <v>743576.044934</v>
+        <v>3566221.084072</v>
       </c>
       <c r="P94" t="n">
-        <v>760004.434981</v>
+        <v>3461618.328436</v>
       </c>
       <c r="Q94" t="n">
-        <v>769929.149969</v>
+        <v>3345848.085239</v>
       </c>
       <c r="R94" t="n">
-        <v>772658.5446</v>
+        <v>3213194.755348</v>
       </c>
       <c r="S94" t="n">
-        <v>769842.683096</v>
+        <v>3069351.334149</v>
       </c>
       <c r="T94" t="n">
-        <v>762849.792616</v>
+        <v>2918336.165959</v>
       </c>
       <c r="U94" t="n">
-        <v>754958.608133</v>
+        <v>2774058.281746</v>
       </c>
       <c r="V94" t="n">
-        <v>748339.797125</v>
+        <v>2647001.957652</v>
       </c>
     </row>
     <row r="95">
@@ -7594,58 +7594,58 @@
         </is>
       </c>
       <c r="E95" t="n">
-        <v>2066012.65503</v>
+        <v>1066221.643942</v>
       </c>
       <c r="F95" t="n">
-        <v>2440888.004758</v>
+        <v>1240042.799019</v>
       </c>
       <c r="G95" t="n">
-        <v>2720445.103232</v>
+        <v>1373548.271721</v>
       </c>
       <c r="H95" t="n">
-        <v>2851792.538358</v>
+        <v>1447447.818611</v>
       </c>
       <c r="I95" t="n">
-        <v>2919171.785713</v>
+        <v>1499523.758869</v>
       </c>
       <c r="J95" t="n">
-        <v>2903163.598192</v>
+        <v>1511230.037192</v>
       </c>
       <c r="K95" t="n">
-        <v>2832860.246904</v>
+        <v>1491251.961611</v>
       </c>
       <c r="L95" t="n">
-        <v>2730842.506047</v>
+        <v>1450594.635092</v>
       </c>
       <c r="M95" t="n">
-        <v>2616797.691297</v>
+        <v>1401185.55116</v>
       </c>
       <c r="N95" t="n">
-        <v>2491332.812507</v>
+        <v>1343864.181797</v>
       </c>
       <c r="O95" t="n">
-        <v>2351670.193296</v>
+        <v>1276903.129858</v>
       </c>
       <c r="P95" t="n">
-        <v>2206111.985139</v>
+        <v>1205099.706778</v>
       </c>
       <c r="Q95" t="n">
-        <v>2057174.036797</v>
+        <v>1129988.676351</v>
       </c>
       <c r="R95" t="n">
-        <v>1907463.406941</v>
+        <v>1053816.158942</v>
       </c>
       <c r="S95" t="n">
-        <v>1763097.228007</v>
+        <v>980215.2472709999</v>
       </c>
       <c r="T95" t="n">
-        <v>1622638.88919</v>
+        <v>908093.943541</v>
       </c>
       <c r="U95" t="n">
-        <v>1486913.725194</v>
+        <v>836855.499683</v>
       </c>
       <c r="V95" t="n">
-        <v>1364733.524338</v>
+        <v>771506.775949</v>
       </c>
     </row>
     <row r="96">
@@ -7670,58 +7670,58 @@
         </is>
       </c>
       <c r="E96" t="n">
-        <v>964728.221628</v>
+        <v>497874.060895</v>
       </c>
       <c r="F96" t="n">
-        <v>989314.434475</v>
+        <v>502600.790386</v>
       </c>
       <c r="G96" t="n">
-        <v>954223.003627</v>
+        <v>481785.629826</v>
       </c>
       <c r="H96" t="n">
-        <v>920079.262655</v>
+        <v>466992.848802</v>
       </c>
       <c r="I96" t="n">
-        <v>910540.068917</v>
+        <v>467727.344251</v>
       </c>
       <c r="J96" t="n">
-        <v>908615.886195</v>
+        <v>472976.314646</v>
       </c>
       <c r="K96" t="n">
-        <v>908413.115738</v>
+        <v>478199.671967</v>
       </c>
       <c r="L96" t="n">
-        <v>907606.892369</v>
+        <v>482111.174822</v>
       </c>
       <c r="M96" t="n">
-        <v>904933.3426569999</v>
+        <v>484553.899108</v>
       </c>
       <c r="N96" t="n">
-        <v>899112.3781419999</v>
+        <v>484995.386538</v>
       </c>
       <c r="O96" t="n">
-        <v>887469.359097</v>
+        <v>481875.564658</v>
       </c>
       <c r="P96" t="n">
-        <v>871429.280253</v>
+        <v>476022.603197</v>
       </c>
       <c r="Q96" t="n">
-        <v>852058.475658</v>
+        <v>468028.670332</v>
       </c>
       <c r="R96" t="n">
-        <v>828434.436276</v>
+        <v>457685.108084</v>
       </c>
       <c r="S96" t="n">
-        <v>801094.14498</v>
+        <v>445377.987632</v>
       </c>
       <c r="T96" t="n">
-        <v>770662.6342410001</v>
+        <v>431293.786517</v>
       </c>
       <c r="U96" t="n">
-        <v>740260.241145</v>
+        <v>416628.647313</v>
       </c>
       <c r="V96" t="n">
-        <v>712552.928836</v>
+        <v>402818.134834</v>
       </c>
     </row>
     <row r="97">
@@ -7746,58 +7746,58 @@
         </is>
       </c>
       <c r="E97" t="n">
-        <v>436488.149079</v>
+        <v>225261.501056</v>
       </c>
       <c r="F97" t="n">
-        <v>413070.047728</v>
+        <v>209851.716743</v>
       </c>
       <c r="G97" t="n">
-        <v>386646.111325</v>
+        <v>195216.987598</v>
       </c>
       <c r="H97" t="n">
-        <v>371514.209603</v>
+        <v>188564.709753</v>
       </c>
       <c r="I97" t="n">
-        <v>371851.215591</v>
+        <v>191012.99049</v>
       </c>
       <c r="J97" t="n">
-        <v>376646.380256</v>
+        <v>196061.745744</v>
       </c>
       <c r="K97" t="n">
-        <v>381847.733633</v>
+        <v>201009.274086</v>
       </c>
       <c r="L97" t="n">
-        <v>386206.027355</v>
+        <v>205148.554002</v>
       </c>
       <c r="M97" t="n">
-        <v>389957.992066</v>
+        <v>208806.170175</v>
       </c>
       <c r="N97" t="n">
-        <v>392834.778879</v>
+        <v>211901.270697</v>
       </c>
       <c r="O97" t="n">
-        <v>393670.292356</v>
+        <v>213753.965107</v>
       </c>
       <c r="P97" t="n">
-        <v>392980.84057</v>
+        <v>214667.749838</v>
       </c>
       <c r="Q97" t="n">
-        <v>390656.908977</v>
+        <v>214584.607615</v>
       </c>
       <c r="R97" t="n">
-        <v>386169.093299</v>
+        <v>213346.80871</v>
       </c>
       <c r="S97" t="n">
-        <v>380351.024409</v>
+        <v>211460.7564</v>
       </c>
       <c r="T97" t="n">
-        <v>373169.980539</v>
+        <v>208840.920489</v>
       </c>
       <c r="U97" t="n">
-        <v>365003.875521</v>
+        <v>205429.202421</v>
       </c>
       <c r="V97" t="n">
-        <v>356555.397475</v>
+        <v>201566.752958</v>
       </c>
     </row>
     <row r="98">
@@ -7822,58 +7822,58 @@
         </is>
       </c>
       <c r="E98" t="n">
-        <v>483322.709775</v>
+        <v>1262915.947889</v>
       </c>
       <c r="F98" t="n">
-        <v>517970.263281</v>
+        <v>1239752.755457</v>
       </c>
       <c r="G98" t="n">
-        <v>525571.76247</v>
+        <v>1130399.554069</v>
       </c>
       <c r="H98" t="n">
-        <v>525513.435685</v>
+        <v>1036368.015627</v>
       </c>
       <c r="I98" t="n">
-        <v>528268.486153</v>
+        <v>979768.183408</v>
       </c>
       <c r="J98" t="n">
-        <v>533544.304009</v>
+        <v>952107.7652190001</v>
       </c>
       <c r="K98" t="n">
-        <v>588681.360549</v>
+        <v>943119.443935</v>
       </c>
       <c r="L98" t="n">
-        <v>638984.374845</v>
+        <v>942705.43111</v>
       </c>
       <c r="M98" t="n">
-        <v>682903.003315</v>
+        <v>943936.529205</v>
       </c>
       <c r="N98" t="n">
-        <v>719084.123531</v>
+        <v>942983.584302</v>
       </c>
       <c r="O98" t="n">
-        <v>745454.181961</v>
+        <v>936113.809414</v>
       </c>
       <c r="P98" t="n">
-        <v>763257.929736</v>
+        <v>924205.333333</v>
       </c>
       <c r="Q98" t="n">
-        <v>775459.09248</v>
+        <v>909602.268585</v>
       </c>
       <c r="R98" t="n">
-        <v>781399.686047</v>
+        <v>891616.324857</v>
       </c>
       <c r="S98" t="n">
-        <v>779485.788997</v>
+        <v>868681.9716319999</v>
       </c>
       <c r="T98" t="n">
-        <v>770871.320363</v>
+        <v>841169.89257</v>
       </c>
       <c r="U98" t="n">
-        <v>757126.054792</v>
+        <v>811005.619111</v>
       </c>
       <c r="V98" t="n">
-        <v>740368.688295</v>
+        <v>780273.420673</v>
       </c>
     </row>
     <row r="99">
@@ -7898,58 +7898,58 @@
         </is>
       </c>
       <c r="E99" t="n">
-        <v>621809.651419</v>
+        <v>1906056.663223</v>
       </c>
       <c r="F99" t="n">
-        <v>665465.428118</v>
+        <v>2129956.700761</v>
       </c>
       <c r="G99" t="n">
-        <v>673261.24463</v>
+        <v>2229750.091803</v>
       </c>
       <c r="H99" t="n">
-        <v>673346.218908</v>
+        <v>2264933.322793</v>
       </c>
       <c r="I99" t="n">
-        <v>679404.799657</v>
+        <v>2289938.925516</v>
       </c>
       <c r="J99" t="n">
-        <v>690716.000157</v>
+        <v>2312597.155749</v>
       </c>
       <c r="K99" t="n">
-        <v>767932.5569119999</v>
+        <v>2335483.295993</v>
       </c>
       <c r="L99" t="n">
-        <v>840518.459625</v>
+        <v>2353477.093105</v>
       </c>
       <c r="M99" t="n">
-        <v>906998.257954</v>
+        <v>2364037.684254</v>
       </c>
       <c r="N99" t="n">
-        <v>966093.35518</v>
+        <v>2366505.363372</v>
       </c>
       <c r="O99" t="n">
-        <v>1016284.060671</v>
+        <v>2358039.351762</v>
       </c>
       <c r="P99" t="n">
-        <v>1058146.649979</v>
+        <v>2342160.151321</v>
       </c>
       <c r="Q99" t="n">
-        <v>1093660.014382</v>
+        <v>2322040.359234</v>
       </c>
       <c r="R99" t="n">
-        <v>1121461.938008</v>
+        <v>2293287.139575</v>
       </c>
       <c r="S99" t="n">
-        <v>1141697.402828</v>
+        <v>2254979.929192</v>
       </c>
       <c r="T99" t="n">
-        <v>1152247.377072</v>
+        <v>2206754.033451</v>
       </c>
       <c r="U99" t="n">
-        <v>1154724.850707</v>
+        <v>2151484.108027</v>
       </c>
       <c r="V99" t="n">
-        <v>1151576.105009</v>
+        <v>2092089.478465</v>
       </c>
     </row>
     <row r="100">
@@ -7974,58 +7974,58 @@
         </is>
       </c>
       <c r="E100" t="n">
-        <v>323610.193625</v>
+        <v>638228.024221</v>
       </c>
       <c r="F100" t="n">
-        <v>349561.104632</v>
+        <v>628364.418125</v>
       </c>
       <c r="G100" t="n">
-        <v>357776.934965</v>
+        <v>587885.941995</v>
       </c>
       <c r="H100" t="n">
-        <v>361260.156769</v>
+        <v>554758.351671</v>
       </c>
       <c r="I100" t="n">
-        <v>366858.302237</v>
+        <v>538635.38514</v>
       </c>
       <c r="J100" t="n">
-        <v>374264.392544</v>
+        <v>535254.583886</v>
       </c>
       <c r="K100" t="n">
-        <v>417173.404587</v>
+        <v>540809.104542</v>
       </c>
       <c r="L100" t="n">
-        <v>458248.148049</v>
+        <v>550848.169862</v>
       </c>
       <c r="M100" t="n">
-        <v>497145.406503</v>
+        <v>562807.66209</v>
       </c>
       <c r="N100" t="n">
-        <v>532936.4821810001</v>
+        <v>575080.339762</v>
       </c>
       <c r="O100" t="n">
-        <v>564791.910174</v>
+        <v>586379.567358</v>
       </c>
       <c r="P100" t="n">
-        <v>593925.173637</v>
+        <v>597746.540898</v>
       </c>
       <c r="Q100" t="n">
-        <v>621033.298317</v>
+        <v>609593.595604</v>
       </c>
       <c r="R100" t="n">
-        <v>644150.523865</v>
+        <v>619613.307252</v>
       </c>
       <c r="S100" t="n">
-        <v>663885.918787</v>
+        <v>626973.783497</v>
       </c>
       <c r="T100" t="n">
-        <v>679985.6777999999</v>
+        <v>631797.479966</v>
       </c>
       <c r="U100" t="n">
-        <v>691127.337249</v>
+        <v>633557.790356</v>
       </c>
       <c r="V100" t="n">
-        <v>698627.820494</v>
+        <v>632892.283308</v>
       </c>
     </row>
     <row r="101">
@@ -8050,58 +8050,58 @@
         </is>
       </c>
       <c r="E101" t="n">
-        <v>312671.353766</v>
+        <v>1125387.735135</v>
       </c>
       <c r="F101" t="n">
-        <v>336179.722459</v>
+        <v>1160796.165596</v>
       </c>
       <c r="G101" t="n">
-        <v>341664.788496</v>
+        <v>1122983.754285</v>
       </c>
       <c r="H101" t="n">
-        <v>342285.166778</v>
+        <v>1074209.536681</v>
       </c>
       <c r="I101" t="n">
-        <v>345000.846207</v>
+        <v>1041480.493579</v>
       </c>
       <c r="J101" t="n">
-        <v>349800.097653</v>
+        <v>1024205.842193</v>
       </c>
       <c r="K101" t="n">
-        <v>387977.728475</v>
+        <v>1018730.070741</v>
       </c>
       <c r="L101" t="n">
-        <v>424430.046263</v>
+        <v>1019129.912801</v>
       </c>
       <c r="M101" t="n">
-        <v>458845.591476</v>
+        <v>1021844.862222</v>
       </c>
       <c r="N101" t="n">
-        <v>490443.159404</v>
+        <v>1025483.130705</v>
       </c>
       <c r="O101" t="n">
-        <v>518547.077519</v>
+        <v>1028397.521667</v>
       </c>
       <c r="P101" t="n">
-        <v>543259.740842</v>
+        <v>1031207.773966</v>
       </c>
       <c r="Q101" t="n">
-        <v>565654.140032</v>
+        <v>1034249.817721</v>
       </c>
       <c r="R101" t="n">
-        <v>584796.182672</v>
+        <v>1034470.800299</v>
       </c>
       <c r="S101" t="n">
-        <v>600688.5888800001</v>
+        <v>1030033.688894</v>
       </c>
       <c r="T101" t="n">
-        <v>612159.187666</v>
+        <v>1020799.240653</v>
       </c>
       <c r="U101" t="n">
-        <v>619944.1793280001</v>
+        <v>1008454.437932</v>
       </c>
       <c r="V101" t="n">
-        <v>625422.101561</v>
+        <v>994509.5229409999</v>
       </c>
     </row>
     <row r="102">
@@ -8126,58 +8126,58 @@
         </is>
       </c>
       <c r="E102" t="n">
-        <v>3687522.570716</v>
+        <v>7305761.376074</v>
       </c>
       <c r="F102" t="n">
-        <v>3973736.200211</v>
+        <v>8099334.653399</v>
       </c>
       <c r="G102" t="n">
-        <v>4043167.461945</v>
+        <v>8445438.616211001</v>
       </c>
       <c r="H102" t="n">
-        <v>4061411.658037</v>
+        <v>8615422.673009999</v>
       </c>
       <c r="I102" t="n">
-        <v>4113948.353787</v>
+        <v>8805331.577624001</v>
       </c>
       <c r="J102" t="n">
-        <v>4195273.319985</v>
+        <v>9023510.958145</v>
       </c>
       <c r="K102" t="n">
-        <v>4674557.775659</v>
+        <v>9259455.323936</v>
       </c>
       <c r="L102" t="n">
-        <v>5124867.676841</v>
+        <v>9479807.172938</v>
       </c>
       <c r="M102" t="n">
-        <v>5539726.973994</v>
+        <v>9659205.947442001</v>
       </c>
       <c r="N102" t="n">
-        <v>5913171.331838</v>
+        <v>9787895.054541999</v>
       </c>
       <c r="O102" t="n">
-        <v>6224854.974864</v>
+        <v>9846848.758165</v>
       </c>
       <c r="P102" t="n">
-        <v>6495377.592179</v>
+        <v>9867482.538000001</v>
       </c>
       <c r="Q102" t="n">
-        <v>6739672.360662</v>
+        <v>9875216.630613999</v>
       </c>
       <c r="R102" t="n">
-        <v>6942372.315292</v>
+        <v>9851990.547792999</v>
       </c>
       <c r="S102" t="n">
-        <v>7092034.01266</v>
+        <v>9784979.004775001</v>
       </c>
       <c r="T102" t="n">
-        <v>7193860.249482</v>
+        <v>9676581.659138</v>
       </c>
       <c r="U102" t="n">
-        <v>7256422.116765</v>
+        <v>9538188.305059001</v>
       </c>
       <c r="V102" t="n">
-        <v>7292667.179766</v>
+        <v>9386269.843513001</v>
       </c>
     </row>
     <row r="103">
@@ -8202,58 +8202,58 @@
         </is>
       </c>
       <c r="E103" t="n">
-        <v>4690128.206769</v>
+        <v>10383212.826496</v>
       </c>
       <c r="F103" t="n">
-        <v>4946086.692704</v>
+        <v>9902748.376832001</v>
       </c>
       <c r="G103" t="n">
-        <v>4936266.865059</v>
+        <v>8862692.386011001</v>
       </c>
       <c r="H103" t="n">
-        <v>4856176.513366</v>
+        <v>8033155.068688</v>
       </c>
       <c r="I103" t="n">
-        <v>4806785.126015</v>
+        <v>7548428.035414</v>
       </c>
       <c r="J103" t="n">
-        <v>4784596.981256</v>
+        <v>7306893.889619</v>
       </c>
       <c r="K103" t="n">
-        <v>5204185.324805</v>
+        <v>7219746.365534</v>
       </c>
       <c r="L103" t="n">
-        <v>5570643.916826</v>
+        <v>7202181.805957</v>
       </c>
       <c r="M103" t="n">
-        <v>5876534.605555</v>
+        <v>7200132.424541</v>
       </c>
       <c r="N103" t="n">
-        <v>6117990.153366</v>
+        <v>7183303.084001</v>
       </c>
       <c r="O103" t="n">
-        <v>6291356.671969</v>
+        <v>7133129.758989</v>
       </c>
       <c r="P103" t="n">
-        <v>6411198.685061</v>
+        <v>7060523.588791</v>
       </c>
       <c r="Q103" t="n">
-        <v>6487382.80424</v>
+        <v>6975245.455563</v>
       </c>
       <c r="R103" t="n">
-        <v>6515140.873039</v>
+        <v>6871138.769377</v>
       </c>
       <c r="S103" t="n">
-        <v>6482417.044303</v>
+        <v>6727840.121151</v>
       </c>
       <c r="T103" t="n">
-        <v>6393238.201274</v>
+        <v>6544677.037276</v>
       </c>
       <c r="U103" t="n">
-        <v>6263265.048437</v>
+        <v>6333398.232627</v>
       </c>
       <c r="V103" t="n">
-        <v>6110113.561196</v>
+        <v>6116846.944304</v>
       </c>
     </row>
     <row r="104">
@@ -8278,58 +8278,58 @@
         </is>
       </c>
       <c r="E104" t="n">
-        <v>4139506.356015</v>
+        <v>801352.713378</v>
       </c>
       <c r="F104" t="n">
-        <v>4342115.134773</v>
+        <v>875765.551586</v>
       </c>
       <c r="G104" t="n">
-        <v>4296081.311526</v>
+        <v>891445.40371</v>
       </c>
       <c r="H104" t="n">
-        <v>4198323.482225</v>
+        <v>897835.398363</v>
       </c>
       <c r="I104" t="n">
-        <v>4145213.299508</v>
+        <v>910995.666078</v>
       </c>
       <c r="J104" t="n">
-        <v>4126759.236588</v>
+        <v>928609.139984</v>
       </c>
       <c r="K104" t="n">
-        <v>3852471.543102</v>
+        <v>947190.63221</v>
       </c>
       <c r="L104" t="n">
-        <v>3613269.832672</v>
+        <v>961707.419214</v>
       </c>
       <c r="M104" t="n">
-        <v>3392910.450571</v>
+        <v>969562.428753</v>
       </c>
       <c r="N104" t="n">
-        <v>3184042.454739</v>
+        <v>969896.887194</v>
       </c>
       <c r="O104" t="n">
-        <v>2980763.950968</v>
+        <v>961478.747369</v>
       </c>
       <c r="P104" t="n">
-        <v>2783002.722383</v>
+        <v>946248.372299</v>
       </c>
       <c r="Q104" t="n">
-        <v>2595639.108183</v>
+        <v>926315.885869</v>
       </c>
       <c r="R104" t="n">
-        <v>2416090.192105</v>
+        <v>901732.479371</v>
       </c>
       <c r="S104" t="n">
-        <v>2241493.554435</v>
+        <v>872648.30175</v>
       </c>
       <c r="T104" t="n">
-        <v>2074093.205839</v>
+        <v>841401.730397</v>
       </c>
       <c r="U104" t="n">
-        <v>1917000.475187</v>
+        <v>810084.938497</v>
       </c>
       <c r="V104" t="n">
-        <v>1772207.441009</v>
+        <v>779603.6700179999</v>
       </c>
     </row>
     <row r="105">
@@ -8354,58 +8354,58 @@
         </is>
       </c>
       <c r="E105" t="n">
-        <v>270639.245254</v>
+        <v>502811.193992</v>
       </c>
       <c r="F105" t="n">
-        <v>300141.922718</v>
+        <v>545653.429629</v>
       </c>
       <c r="G105" t="n">
-        <v>312256.660638</v>
+        <v>561683.291014</v>
       </c>
       <c r="H105" t="n">
-        <v>319541.288537</v>
+        <v>566997.8252739999</v>
       </c>
       <c r="I105" t="n">
-        <v>329314.65591</v>
+        <v>574611.060913</v>
       </c>
       <c r="J105" t="n">
-        <v>341640.353555</v>
+        <v>584596.584391</v>
       </c>
       <c r="K105" t="n">
-        <v>387075.664859</v>
+        <v>597672.405604</v>
       </c>
       <c r="L105" t="n">
-        <v>430677.238656</v>
+        <v>612054.237757</v>
       </c>
       <c r="M105" t="n">
-        <v>471030.188816</v>
+        <v>626264.866283</v>
       </c>
       <c r="N105" t="n">
-        <v>507174.714925</v>
+        <v>638621.271389</v>
       </c>
       <c r="O105" t="n">
-        <v>538518.146675</v>
+        <v>647223.516605</v>
       </c>
       <c r="P105" t="n">
-        <v>566594.757471</v>
+        <v>653136.3999120001</v>
       </c>
       <c r="Q105" t="n">
-        <v>591019.674336</v>
+        <v>656664.4521080001</v>
       </c>
       <c r="R105" t="n">
-        <v>610864.918242</v>
+        <v>656602.905129</v>
       </c>
       <c r="S105" t="n">
-        <v>626779.170182</v>
+        <v>653217.4929289999</v>
       </c>
       <c r="T105" t="n">
-        <v>637586.234143</v>
+        <v>646887.75786</v>
       </c>
       <c r="U105" t="n">
-        <v>644037.444685</v>
+        <v>638732.573642</v>
       </c>
       <c r="V105" t="n">
-        <v>647319.2428520001</v>
+        <v>629181.388571</v>
       </c>
     </row>
     <row r="106">
@@ -8430,58 +8430,58 @@
         </is>
       </c>
       <c r="E106" t="n">
-        <v>3529656.875241</v>
+        <v>5679399.873843</v>
       </c>
       <c r="F106" t="n">
-        <v>3704262.146675</v>
+        <v>6368288.695843</v>
       </c>
       <c r="G106" t="n">
-        <v>3665390.939909</v>
+        <v>6740621.899</v>
       </c>
       <c r="H106" t="n">
-        <v>3587255.347871</v>
+        <v>6896417.277492</v>
       </c>
       <c r="I106" t="n">
-        <v>3547225.911731</v>
+        <v>6996307.983777</v>
       </c>
       <c r="J106" t="n">
-        <v>3536866.189316</v>
+        <v>7062117.261531</v>
       </c>
       <c r="K106" t="n">
-        <v>3855597.342406</v>
+        <v>7100983.23676</v>
       </c>
       <c r="L106" t="n">
-        <v>4134358.507372</v>
+        <v>7093686.751449</v>
       </c>
       <c r="M106" t="n">
-        <v>4367085.116687</v>
+        <v>7041712.602556</v>
       </c>
       <c r="N106" t="n">
-        <v>4549054.181146</v>
+        <v>6946348.421262</v>
       </c>
       <c r="O106" t="n">
-        <v>4665493.661058</v>
+        <v>6794529.930177</v>
       </c>
       <c r="P106" t="n">
-        <v>4729395.661344</v>
+        <v>6602294.14067</v>
       </c>
       <c r="Q106" t="n">
-        <v>4760868.838741</v>
+        <v>6392813.744478</v>
       </c>
       <c r="R106" t="n">
-        <v>4759968.657589</v>
+        <v>6168048.339403</v>
       </c>
       <c r="S106" t="n">
-        <v>4721412.058817</v>
+        <v>5931534.832286</v>
       </c>
       <c r="T106" t="n">
-        <v>4654611.592467</v>
+        <v>5695486.181198</v>
       </c>
       <c r="U106" t="n">
-        <v>4566413.077023</v>
+        <v>5465156.876537</v>
       </c>
       <c r="V106" t="n">
-        <v>4464115.488387</v>
+        <v>5240530.639098</v>
       </c>
     </row>
     <row r="107">
@@ -8506,58 +8506,58 @@
         </is>
       </c>
       <c r="E107" t="n">
-        <v>29582.687546</v>
+        <v>163792.791879</v>
       </c>
       <c r="F107" t="n">
-        <v>32942.656436</v>
+        <v>188134.146929</v>
       </c>
       <c r="G107" t="n">
-        <v>34853.492428</v>
+        <v>193028.143751</v>
       </c>
       <c r="H107" t="n">
-        <v>36367.293842</v>
+        <v>193443.593758</v>
       </c>
       <c r="I107" t="n">
-        <v>38141.456677</v>
+        <v>196173.869446</v>
       </c>
       <c r="J107" t="n">
-        <v>40137.397889</v>
+        <v>201615.670699</v>
       </c>
       <c r="K107" t="n">
-        <v>46010.612346</v>
+        <v>208916.232962</v>
       </c>
       <c r="L107" t="n">
-        <v>51744.128384</v>
+        <v>216513.981995</v>
       </c>
       <c r="M107" t="n">
-        <v>57187.376937</v>
+        <v>223154.031922</v>
       </c>
       <c r="N107" t="n">
-        <v>62196.616147</v>
+        <v>228049.314376</v>
       </c>
       <c r="O107" t="n">
-        <v>66564.813243</v>
+        <v>230622.360452</v>
       </c>
       <c r="P107" t="n">
-        <v>70342.38735999999</v>
+        <v>231328.391795</v>
       </c>
       <c r="Q107" t="n">
-        <v>73503.821992</v>
+        <v>230437.786498</v>
       </c>
       <c r="R107" t="n">
-        <v>75911.247661</v>
+        <v>227587.295343</v>
       </c>
       <c r="S107" t="n">
-        <v>77517.694458</v>
+        <v>222666.002218</v>
       </c>
       <c r="T107" t="n">
-        <v>78269.765462</v>
+        <v>215885.594646</v>
       </c>
       <c r="U107" t="n">
-        <v>78284.526444</v>
+        <v>207880.812653</v>
       </c>
       <c r="V107" t="n">
-        <v>77738.070894</v>
+        <v>199187.810941</v>
       </c>
     </row>
     <row r="108">
@@ -8582,58 +8582,58 @@
         </is>
       </c>
       <c r="E108" t="n">
-        <v>948451.299522</v>
+        <v>2597978.257416</v>
       </c>
       <c r="F108" t="n">
-        <v>1012895.603406</v>
+        <v>2738165.87567</v>
       </c>
       <c r="G108" t="n">
-        <v>1024898.694472</v>
+        <v>2670376.375637</v>
       </c>
       <c r="H108" t="n">
-        <v>1023820.212298</v>
+        <v>2571054.167711</v>
       </c>
       <c r="I108" t="n">
-        <v>1029215.76169</v>
+        <v>2506626.307414</v>
       </c>
       <c r="J108" t="n">
-        <v>1039442.262225</v>
+        <v>2477212.656844</v>
       </c>
       <c r="K108" t="n">
-        <v>1146090.65187</v>
+        <v>2472590.487582</v>
       </c>
       <c r="L108" t="n">
-        <v>1244042.239568</v>
+        <v>2478232.297304</v>
       </c>
       <c r="M108" t="n">
-        <v>1332807.601407</v>
+        <v>2483402.69732</v>
       </c>
       <c r="N108" t="n">
-        <v>1411290.475183</v>
+        <v>2483367.390313</v>
       </c>
       <c r="O108" t="n">
-        <v>1478810.125013</v>
+        <v>2475204.471255</v>
       </c>
       <c r="P108" t="n">
-        <v>1538068.934539</v>
+        <v>2465086.289378</v>
       </c>
       <c r="Q108" t="n">
-        <v>1588845.908651</v>
+        <v>2454666.940135</v>
       </c>
       <c r="R108" t="n">
-        <v>1629650.406599</v>
+        <v>2438428.196294</v>
       </c>
       <c r="S108" t="n">
-        <v>1657811.381998</v>
+        <v>2411762.996701</v>
       </c>
       <c r="T108" t="n">
-        <v>1673221.31066</v>
+        <v>2373178.972734</v>
       </c>
       <c r="U108" t="n">
-        <v>1677720.377755</v>
+        <v>2323959.416109</v>
       </c>
       <c r="V108" t="n">
-        <v>1674770.603879</v>
+        <v>2268669.935721</v>
       </c>
     </row>
     <row r="109">
@@ -8658,58 +8658,58 @@
         </is>
       </c>
       <c r="E109" t="n">
-        <v>4001616.432705</v>
+        <v>790270.0610399999</v>
       </c>
       <c r="F109" t="n">
-        <v>4245116.550768</v>
+        <v>867537.860475</v>
       </c>
       <c r="G109" t="n">
-        <v>4230114.825888</v>
+        <v>920475.091362</v>
       </c>
       <c r="H109" t="n">
-        <v>4157416.098459</v>
+        <v>970798.416075</v>
       </c>
       <c r="I109" t="n">
-        <v>4123468.708552</v>
+        <v>1030323.241959</v>
       </c>
       <c r="J109" t="n">
-        <v>4122840.466211</v>
+        <v>1087694.962397</v>
       </c>
       <c r="K109" t="n">
-        <v>3865403.101178</v>
+        <v>1137998.487029</v>
       </c>
       <c r="L109" t="n">
-        <v>3643187.744053</v>
+        <v>1176029.172721</v>
       </c>
       <c r="M109" t="n">
-        <v>3440127.521934</v>
+        <v>1200131.650734</v>
       </c>
       <c r="N109" t="n">
-        <v>3247775.714482</v>
+        <v>1211269.149094</v>
       </c>
       <c r="O109" t="n">
-        <v>3058579.990376</v>
+        <v>1209501.762396</v>
       </c>
       <c r="P109" t="n">
-        <v>2875967.49811</v>
+        <v>1198828.428475</v>
       </c>
       <c r="Q109" t="n">
-        <v>2697201.140533</v>
+        <v>1181044.674642</v>
       </c>
       <c r="R109" t="n">
-        <v>2521435.957587</v>
+        <v>1154873.5438</v>
       </c>
       <c r="S109" t="n">
-        <v>2354304.76901</v>
+        <v>1122438.587408</v>
       </c>
       <c r="T109" t="n">
-        <v>2191593.472558</v>
+        <v>1085953.873553</v>
       </c>
       <c r="U109" t="n">
-        <v>2034585.755151</v>
+        <v>1047855.636496</v>
       </c>
       <c r="V109" t="n">
-        <v>1886476.596152</v>
+        <v>1009179.2877</v>
       </c>
     </row>
     <row r="110">
@@ -8734,58 +8734,58 @@
         </is>
       </c>
       <c r="E110" t="n">
-        <v>552189.55105</v>
+        <v>1503973.810546</v>
       </c>
       <c r="F110" t="n">
-        <v>602087.010516</v>
+        <v>1679119.819242</v>
       </c>
       <c r="G110" t="n">
-        <v>620441.163441</v>
+        <v>1763587.695305</v>
       </c>
       <c r="H110" t="n">
-        <v>629838.535635</v>
+        <v>1796450.273417</v>
       </c>
       <c r="I110" t="n">
-        <v>643783.470648</v>
+        <v>1820142.964196</v>
       </c>
       <c r="J110" t="n">
-        <v>663362.946524</v>
+        <v>1846350.246921</v>
       </c>
       <c r="K110" t="n">
-        <v>749232.553979</v>
+        <v>1878744.662039</v>
       </c>
       <c r="L110" t="n">
-        <v>834704.8811689999</v>
+        <v>1913811.449858</v>
       </c>
       <c r="M110" t="n">
-        <v>917448.814378</v>
+        <v>1949412.443872</v>
       </c>
       <c r="N110" t="n">
-        <v>994620.526012</v>
+        <v>1983966.548643</v>
       </c>
       <c r="O110" t="n">
-        <v>1063661.602185</v>
+        <v>2012289.734185</v>
       </c>
       <c r="P110" t="n">
-        <v>1126334.816028</v>
+        <v>2035476.888589</v>
       </c>
       <c r="Q110" t="n">
-        <v>1184011.922915</v>
+        <v>2053759.516483</v>
       </c>
       <c r="R110" t="n">
-        <v>1234262.915075</v>
+        <v>2061955.565019</v>
       </c>
       <c r="S110" t="n">
-        <v>1273768.569692</v>
+        <v>2057023.201603</v>
       </c>
       <c r="T110" t="n">
-        <v>1302455.082836</v>
+        <v>2040739.003482</v>
       </c>
       <c r="U110" t="n">
-        <v>1322052.821164</v>
+        <v>2015501.983304</v>
       </c>
       <c r="V110" t="n">
-        <v>1335853.153561</v>
+        <v>1985336.519301</v>
       </c>
     </row>
     <row r="111">
@@ -8810,58 +8810,58 @@
         </is>
       </c>
       <c r="E111" t="n">
-        <v>17260014.721263</v>
+        <v>3865461.172719</v>
       </c>
       <c r="F111" t="n">
-        <v>18472159.532676</v>
+        <v>4312766.424521</v>
       </c>
       <c r="G111" t="n">
-        <v>18587561.919627</v>
+        <v>4448448.520134</v>
       </c>
       <c r="H111" t="n">
-        <v>18461647.941216</v>
+        <v>4472165.904696</v>
       </c>
       <c r="I111" t="n">
-        <v>18530203.585594</v>
+        <v>4521064.155805</v>
       </c>
       <c r="J111" t="n">
-        <v>18766131.398067</v>
+        <v>4599720.751588</v>
       </c>
       <c r="K111" t="n">
-        <v>17803520.305734</v>
+        <v>4694716.371073</v>
       </c>
       <c r="L111" t="n">
-        <v>16932077.937377</v>
+        <v>4779664.9461</v>
       </c>
       <c r="M111" t="n">
-        <v>16081623.057578</v>
+        <v>4842448.841547</v>
       </c>
       <c r="N111" t="n">
-        <v>15233383.285615</v>
+        <v>4872517.561609</v>
       </c>
       <c r="O111" t="n">
-        <v>14356234.045994</v>
+        <v>4852594.857227</v>
       </c>
       <c r="P111" t="n">
-        <v>13477343.91227</v>
+        <v>4787937.075235</v>
       </c>
       <c r="Q111" t="n">
-        <v>12632908.168991</v>
+        <v>4692424.061603</v>
       </c>
       <c r="R111" t="n">
-        <v>11802103.892598</v>
+        <v>4566160.22081</v>
       </c>
       <c r="S111" t="n">
-        <v>10976199.525089</v>
+        <v>4412695.638067</v>
       </c>
       <c r="T111" t="n">
-        <v>10188885.41619</v>
+        <v>4251949.353955</v>
       </c>
       <c r="U111" t="n">
-        <v>9456503.83735</v>
+        <v>4097545.525643</v>
       </c>
       <c r="V111" t="n">
-        <v>8781821.078677</v>
+        <v>3950285.771741</v>
       </c>
     </row>
     <row r="112">
@@ -8886,58 +8886,58 @@
         </is>
       </c>
       <c r="E112" t="n">
-        <v>3637394.330133</v>
+        <v>5961513.73695</v>
       </c>
       <c r="F112" t="n">
-        <v>3923657.593469</v>
+        <v>6687992.688776</v>
       </c>
       <c r="G112" t="n">
-        <v>3993131.532569</v>
+        <v>7073622.833779</v>
       </c>
       <c r="H112" t="n">
-        <v>4008059.240355</v>
+        <v>7298252.764724</v>
       </c>
       <c r="I112" t="n">
-        <v>4054063.41895</v>
+        <v>7521068.333045</v>
       </c>
       <c r="J112" t="n">
-        <v>4130465.248177</v>
+        <v>7753353.124989</v>
       </c>
       <c r="K112" t="n">
-        <v>4605583.756779</v>
+        <v>7995337.563303</v>
       </c>
       <c r="L112" t="n">
-        <v>5059089.764574</v>
+        <v>8220995.054102</v>
       </c>
       <c r="M112" t="n">
-        <v>5479416.82602</v>
+        <v>8413736.120384</v>
       </c>
       <c r="N112" t="n">
-        <v>5855355.40101</v>
+        <v>8569324.874194</v>
       </c>
       <c r="O112" t="n">
-        <v>6181102.817032</v>
+        <v>8678663.882679</v>
       </c>
       <c r="P112" t="n">
-        <v>6474061.747192</v>
+        <v>8762616.295472</v>
       </c>
       <c r="Q112" t="n">
-        <v>6734848.5137</v>
+        <v>8827633.619016999</v>
       </c>
       <c r="R112" t="n">
-        <v>6954005.539214</v>
+        <v>8856109.81127</v>
       </c>
       <c r="S112" t="n">
-        <v>7127910.165615</v>
+        <v>8839930.093649</v>
       </c>
       <c r="T112" t="n">
-        <v>7244590.88273</v>
+        <v>8774407.165663</v>
       </c>
       <c r="U112" t="n">
-        <v>7314576.161011</v>
+        <v>8670977.807057001</v>
       </c>
       <c r="V112" t="n">
-        <v>7354615.524202</v>
+        <v>8548836.139638999</v>
       </c>
     </row>
     <row r="113">
@@ -9190,58 +9190,58 @@
         </is>
       </c>
       <c r="E116" t="n">
-        <v>436872.892377</v>
+        <v>92500.424767</v>
       </c>
       <c r="F116" t="n">
-        <v>454263.044157</v>
+        <v>103953.439117</v>
       </c>
       <c r="G116" t="n">
-        <v>448880.541358</v>
+        <v>107318.569526</v>
       </c>
       <c r="H116" t="n">
-        <v>451459.77922</v>
+        <v>110452.673162</v>
       </c>
       <c r="I116" t="n">
-        <v>460615.710433</v>
+        <v>113646.888845</v>
       </c>
       <c r="J116" t="n">
-        <v>471461.435406</v>
+        <v>116328.186314</v>
       </c>
       <c r="K116" t="n">
-        <v>479586.057545</v>
+        <v>117952.406426</v>
       </c>
       <c r="L116" t="n">
-        <v>491607.425753</v>
+        <v>118110.137669</v>
       </c>
       <c r="M116" t="n">
-        <v>502571.275504</v>
+        <v>117243.214733</v>
       </c>
       <c r="N116" t="n">
-        <v>503907.67816</v>
+        <v>115104.335349</v>
       </c>
       <c r="O116" t="n">
-        <v>493573.694657</v>
+        <v>111623.254198</v>
       </c>
       <c r="P116" t="n">
-        <v>477343.379868</v>
+        <v>107443.689261</v>
       </c>
       <c r="Q116" t="n">
-        <v>458985.028436</v>
+        <v>102937.99314</v>
       </c>
       <c r="R116" t="n">
-        <v>437841.330568</v>
+        <v>97832.93438000001</v>
       </c>
       <c r="S116" t="n">
-        <v>413317.672896</v>
+        <v>91974.76863799999</v>
       </c>
       <c r="T116" t="n">
-        <v>386292.957897</v>
+        <v>85584.763332</v>
       </c>
       <c r="U116" t="n">
-        <v>358064.047947</v>
+        <v>79017.052039</v>
       </c>
       <c r="V116" t="n">
-        <v>328589.998865</v>
+        <v>72333.139297</v>
       </c>
     </row>
     <row r="117">
@@ -9266,58 +9266,58 @@
         </is>
       </c>
       <c r="E117" t="n">
-        <v>724526.425051</v>
+        <v>153406.181161</v>
       </c>
       <c r="F117" t="n">
-        <v>892258.252705</v>
+        <v>204184.150883</v>
       </c>
       <c r="G117" t="n">
-        <v>930256.774716</v>
+        <v>222406.224276</v>
       </c>
       <c r="H117" t="n">
-        <v>948807.853491</v>
+        <v>232132.226521</v>
       </c>
       <c r="I117" t="n">
-        <v>964755.362417</v>
+        <v>238032.361798</v>
       </c>
       <c r="J117" t="n">
-        <v>975602.192057</v>
+        <v>240719.653917</v>
       </c>
       <c r="K117" t="n">
-        <v>976435.964697</v>
+        <v>240150.792427</v>
       </c>
       <c r="L117" t="n">
-        <v>960725.5003439999</v>
+        <v>230817.142224</v>
       </c>
       <c r="M117" t="n">
-        <v>931926.1419019999</v>
+        <v>217406.012034</v>
       </c>
       <c r="N117" t="n">
-        <v>890758.701159</v>
+        <v>203470.184514</v>
       </c>
       <c r="O117" t="n">
-        <v>841258.912717</v>
+        <v>190253.367385</v>
       </c>
       <c r="P117" t="n">
-        <v>789782.572649</v>
+        <v>177769.624339</v>
       </c>
       <c r="Q117" t="n">
-        <v>739493.26464</v>
+        <v>165848.443602</v>
       </c>
       <c r="R117" t="n">
-        <v>690268.9816300001</v>
+        <v>154236.330081</v>
       </c>
       <c r="S117" t="n">
-        <v>641442.212907</v>
+        <v>142738.873742</v>
       </c>
       <c r="T117" t="n">
-        <v>592195.2463070001</v>
+        <v>131203.246047</v>
       </c>
       <c r="U117" t="n">
-        <v>543802.587956</v>
+        <v>120005.562239</v>
       </c>
       <c r="V117" t="n">
-        <v>498613.803791</v>
+        <v>109760.801757</v>
       </c>
     </row>
     <row r="118">
@@ -9342,58 +9342,58 @@
         </is>
       </c>
       <c r="E118" t="n">
-        <v>1488772.754535</v>
+        <v>315222.37836</v>
       </c>
       <c r="F118" t="n">
-        <v>1447956.273684</v>
+        <v>331349.944214</v>
       </c>
       <c r="G118" t="n">
-        <v>1331325.351123</v>
+        <v>318293.886886</v>
       </c>
       <c r="H118" t="n">
-        <v>1263700.382458</v>
+        <v>309172.802856</v>
       </c>
       <c r="I118" t="n">
-        <v>1235189.614701</v>
+        <v>304756.120266</v>
       </c>
       <c r="J118" t="n">
-        <v>1221800.886511</v>
+        <v>301466.611033</v>
       </c>
       <c r="K118" t="n">
-        <v>1207244.264674</v>
+        <v>296917.235023</v>
       </c>
       <c r="L118" t="n">
-        <v>1180706.829551</v>
+        <v>283668.307027</v>
       </c>
       <c r="M118" t="n">
-        <v>1146291.803893</v>
+        <v>267414.678595</v>
       </c>
       <c r="N118" t="n">
-        <v>1103989.679244</v>
+        <v>252177.1423</v>
       </c>
       <c r="O118" t="n">
-        <v>1055399.90383</v>
+        <v>238682.030711</v>
       </c>
       <c r="P118" t="n">
-        <v>1005660.696553</v>
+        <v>226360.938351</v>
       </c>
       <c r="Q118" t="n">
-        <v>957123.164355</v>
+        <v>214656.974896</v>
       </c>
       <c r="R118" t="n">
-        <v>907516.275911</v>
+        <v>202778.892881</v>
       </c>
       <c r="S118" t="n">
-        <v>855684.170534</v>
+        <v>190413.715099</v>
       </c>
       <c r="T118" t="n">
-        <v>802049.2452079999</v>
+        <v>177697.246165</v>
       </c>
       <c r="U118" t="n">
-        <v>748121.89608</v>
+        <v>165094.449255</v>
       </c>
       <c r="V118" t="n">
-        <v>693879.6721110001</v>
+        <v>152745.047479</v>
       </c>
     </row>
     <row r="119">
@@ -9418,58 +9418,58 @@
         </is>
       </c>
       <c r="E119" t="n">
-        <v>406370.672851</v>
+        <v>86042.097158</v>
       </c>
       <c r="F119" t="n">
-        <v>479164.332756</v>
+        <v>109651.843646</v>
       </c>
       <c r="G119" t="n">
-        <v>524343.288569</v>
+        <v>125360.238382</v>
       </c>
       <c r="H119" t="n">
-        <v>569075.381411</v>
+        <v>139228.121752</v>
       </c>
       <c r="I119" t="n">
-        <v>612521.71369</v>
+        <v>151126.384825</v>
       </c>
       <c r="J119" t="n">
-        <v>650395.030495</v>
+        <v>160478.182526</v>
       </c>
       <c r="K119" t="n">
-        <v>678560.578386</v>
+        <v>166889.449489</v>
       </c>
       <c r="L119" t="n">
-        <v>692339.7510479999</v>
+        <v>166336.672366</v>
       </c>
       <c r="M119" t="n">
-        <v>695681.497805</v>
+        <v>162293.269051</v>
       </c>
       <c r="N119" t="n">
-        <v>689264.035438</v>
+        <v>157444.075805</v>
       </c>
       <c r="O119" t="n">
-        <v>673802.0633</v>
+        <v>152382.470552</v>
       </c>
       <c r="P119" t="n">
-        <v>652569.7081629999</v>
+        <v>146884.821079</v>
       </c>
       <c r="Q119" t="n">
-        <v>627844.906613</v>
+        <v>140808.720733</v>
       </c>
       <c r="R119" t="n">
-        <v>600119.90478</v>
+        <v>134093.077025</v>
       </c>
       <c r="S119" t="n">
-        <v>570277.3990419999</v>
+        <v>126902.707713</v>
       </c>
       <c r="T119" t="n">
-        <v>538124.457882</v>
+        <v>119223.644722</v>
       </c>
       <c r="U119" t="n">
-        <v>504105.657523</v>
+        <v>111245.301509</v>
       </c>
       <c r="V119" t="n">
-        <v>469017.675502</v>
+        <v>103245.749937</v>
       </c>
     </row>
     <row r="120">
@@ -9494,58 +9494,58 @@
         </is>
       </c>
       <c r="E120" t="n">
-        <v>147267.556439</v>
+        <v>31181.407139</v>
       </c>
       <c r="F120" t="n">
-        <v>153733.335307</v>
+        <v>35180.297226</v>
       </c>
       <c r="G120" t="n">
-        <v>152987.235459</v>
+        <v>36576.259723</v>
       </c>
       <c r="H120" t="n">
-        <v>155343.951965</v>
+        <v>38005.943262</v>
       </c>
       <c r="I120" t="n">
-        <v>160322.752695</v>
+        <v>39556.145486</v>
       </c>
       <c r="J120" t="n">
-        <v>166210.984202</v>
+        <v>41010.824822</v>
       </c>
       <c r="K120" t="n">
-        <v>171348.874809</v>
+        <v>42142.61821</v>
       </c>
       <c r="L120" t="n">
-        <v>178159.20753</v>
+        <v>42803.276407</v>
       </c>
       <c r="M120" t="n">
-        <v>184844.931002</v>
+        <v>43121.871452</v>
       </c>
       <c r="N120" t="n">
-        <v>188061.99905</v>
+        <v>42957.772511</v>
       </c>
       <c r="O120" t="n">
-        <v>186529.819359</v>
+        <v>42184.30939</v>
       </c>
       <c r="P120" t="n">
-        <v>182356.838316</v>
+        <v>41046.115432</v>
       </c>
       <c r="Q120" t="n">
-        <v>177040.221018</v>
+        <v>39705.358405</v>
       </c>
       <c r="R120" t="n">
-        <v>170680.411317</v>
+        <v>38137.481125</v>
       </c>
       <c r="S120" t="n">
-        <v>162868.374622</v>
+        <v>36242.778997</v>
       </c>
       <c r="T120" t="n">
-        <v>153966.097735</v>
+        <v>34111.810134</v>
       </c>
       <c r="U120" t="n">
-        <v>144331.673554</v>
+        <v>31850.903282</v>
       </c>
       <c r="V120" t="n">
-        <v>133887.098793</v>
+        <v>29472.820842</v>
       </c>
     </row>
     <row r="121">
@@ -9570,58 +9570,58 @@
         </is>
       </c>
       <c r="E121" t="n">
-        <v>1816604.884252</v>
+        <v>384635.271172</v>
       </c>
       <c r="F121" t="n">
-        <v>2118097.191541</v>
+        <v>484704.820866</v>
       </c>
       <c r="G121" t="n">
-        <v>2293278.27637</v>
+        <v>548278.0416380001</v>
       </c>
       <c r="H121" t="n">
-        <v>2436177.165462</v>
+        <v>596027.1382010001</v>
       </c>
       <c r="I121" t="n">
-        <v>2539550.120846</v>
+        <v>626578.650628</v>
       </c>
       <c r="J121" t="n">
-        <v>2597416.212103</v>
+        <v>640885.328822</v>
       </c>
       <c r="K121" t="n">
-        <v>2608759.992207</v>
+        <v>641614.813497</v>
       </c>
       <c r="L121" t="n">
-        <v>2577406.107941</v>
+        <v>619229.438556</v>
       </c>
       <c r="M121" t="n">
-        <v>2527339.509143</v>
+        <v>589594.796232</v>
       </c>
       <c r="N121" t="n">
-        <v>2458278.491623</v>
+        <v>561528.4786180001</v>
       </c>
       <c r="O121" t="n">
-        <v>2369146.351197</v>
+        <v>535789.950428</v>
       </c>
       <c r="P121" t="n">
-        <v>2269413.946924</v>
+        <v>510815.10125</v>
       </c>
       <c r="Q121" t="n">
-        <v>2165240.037821</v>
+        <v>485605.085898</v>
       </c>
       <c r="R121" t="n">
-        <v>2056383.614035</v>
+        <v>459486.186265</v>
       </c>
       <c r="S121" t="n">
-        <v>1944790.692425</v>
+        <v>432770.446838</v>
       </c>
       <c r="T121" t="n">
-        <v>1828723.199524</v>
+        <v>405161.002888</v>
       </c>
       <c r="U121" t="n">
-        <v>1708140.952939</v>
+        <v>376950.055002</v>
       </c>
       <c r="V121" t="n">
-        <v>1585072.233852</v>
+        <v>348924.955361</v>
       </c>
     </row>
     <row r="122">
@@ -9646,58 +9646,58 @@
         </is>
       </c>
       <c r="E122" t="n">
-        <v>269419.679705</v>
+        <v>4226847.105453</v>
       </c>
       <c r="F122" t="n">
-        <v>509796.806557</v>
+        <v>4786244.740755</v>
       </c>
       <c r="G122" t="n">
-        <v>688781.088463</v>
+        <v>5011619.335628</v>
       </c>
       <c r="H122" t="n">
-        <v>858583.194653</v>
+        <v>5258128.802904</v>
       </c>
       <c r="I122" t="n">
-        <v>1038157.049637</v>
+        <v>5537415.772572</v>
       </c>
       <c r="J122" t="n">
-        <v>1225689.744246</v>
+        <v>5807687.697586</v>
       </c>
       <c r="K122" t="n">
-        <v>1410489.852888</v>
+        <v>6026758.270137</v>
       </c>
       <c r="L122" t="n">
-        <v>1583542.678678</v>
+        <v>6203522.526594</v>
       </c>
       <c r="M122" t="n">
-        <v>1735860.930094</v>
+        <v>6327442.247246</v>
       </c>
       <c r="N122" t="n">
-        <v>1852048.511166</v>
+        <v>6353627.106743</v>
       </c>
       <c r="O122" t="n">
-        <v>1929694.180308</v>
+        <v>6278489.542705</v>
       </c>
       <c r="P122" t="n">
-        <v>1981061.237567</v>
+        <v>6147868.090328</v>
       </c>
       <c r="Q122" t="n">
-        <v>2016419.777671</v>
+        <v>5992583.82388</v>
       </c>
       <c r="R122" t="n">
-        <v>2038406.373677</v>
+        <v>5814651.990161</v>
       </c>
       <c r="S122" t="n">
-        <v>2050515.676084</v>
+        <v>5617852.907483</v>
       </c>
       <c r="T122" t="n">
-        <v>2055002.722233</v>
+        <v>5403372.213499</v>
       </c>
       <c r="U122" t="n">
-        <v>2053167.287734</v>
+        <v>5175570.780406</v>
       </c>
       <c r="V122" t="n">
-        <v>2037679.958888</v>
+        <v>4930257.927129</v>
       </c>
     </row>
     <row r="123">
@@ -9722,58 +9722,58 @@
         </is>
       </c>
       <c r="E123" t="n">
-        <v>78751.616077</v>
+        <v>142645.250144</v>
       </c>
       <c r="F123" t="n">
-        <v>87444.91088</v>
+        <v>154207.297679</v>
       </c>
       <c r="G123" t="n">
-        <v>91945.894609</v>
+        <v>162963.523984</v>
       </c>
       <c r="H123" t="n">
-        <v>94885.008843</v>
+        <v>169114.793272</v>
       </c>
       <c r="I123" t="n">
-        <v>97606.43193399999</v>
+        <v>175025.652074</v>
       </c>
       <c r="J123" t="n">
-        <v>100835.433839</v>
+        <v>181638.48104</v>
       </c>
       <c r="K123" t="n">
-        <v>104374.526975</v>
+        <v>188405.692368</v>
       </c>
       <c r="L123" t="n">
-        <v>107999.190421</v>
+        <v>195272.664181</v>
       </c>
       <c r="M123" t="n">
-        <v>111214.193985</v>
+        <v>201462.641186</v>
       </c>
       <c r="N123" t="n">
-        <v>114034.194741</v>
+        <v>206798.291886</v>
       </c>
       <c r="O123" t="n">
-        <v>116026.113181</v>
+        <v>210037.389665</v>
       </c>
       <c r="P123" t="n">
-        <v>117550.42553</v>
+        <v>211787.157029</v>
       </c>
       <c r="Q123" t="n">
-        <v>118594.704635</v>
+        <v>211995.683988</v>
       </c>
       <c r="R123" t="n">
-        <v>118961.893336</v>
+        <v>210537.095805</v>
       </c>
       <c r="S123" t="n">
-        <v>118549.747206</v>
+        <v>207405.148155</v>
       </c>
       <c r="T123" t="n">
-        <v>117513.650498</v>
+        <v>202999.357741</v>
       </c>
       <c r="U123" t="n">
-        <v>115985.735433</v>
+        <v>197734.776308</v>
       </c>
       <c r="V123" t="n">
-        <v>114256.176211</v>
+        <v>192119.726208</v>
       </c>
     </row>
     <row r="124">
@@ -9798,58 +9798,58 @@
         </is>
       </c>
       <c r="E124" t="n">
-        <v>801005.692519</v>
+        <v>1038577.022158</v>
       </c>
       <c r="F124" t="n">
-        <v>875562.389844</v>
+        <v>1140930.404993</v>
       </c>
       <c r="G124" t="n">
-        <v>915129.810867</v>
+        <v>1202474.265463</v>
       </c>
       <c r="H124" t="n">
-        <v>943397.417949</v>
+        <v>1239346.36713</v>
       </c>
       <c r="I124" t="n">
-        <v>971351.789234</v>
+        <v>1267148.208796</v>
       </c>
       <c r="J124" t="n">
-        <v>1004223.076892</v>
+        <v>1295532.324412</v>
       </c>
       <c r="K124" t="n">
-        <v>1040217.711584</v>
+        <v>1324813.494573</v>
       </c>
       <c r="L124" t="n">
-        <v>1078853.028961</v>
+        <v>1355657.493668</v>
       </c>
       <c r="M124" t="n">
-        <v>1116126.435778</v>
+        <v>1383853.566537</v>
       </c>
       <c r="N124" t="n">
-        <v>1151305.382144</v>
+        <v>1409737.77567</v>
       </c>
       <c r="O124" t="n">
-        <v>1178341.247184</v>
+        <v>1425921.984893</v>
       </c>
       <c r="P124" t="n">
-        <v>1199869.963593</v>
+        <v>1437267.953172</v>
       </c>
       <c r="Q124" t="n">
-        <v>1214638.489266</v>
+        <v>1442125.202451</v>
       </c>
       <c r="R124" t="n">
-        <v>1223952.787227</v>
+        <v>1440276.341564</v>
       </c>
       <c r="S124" t="n">
-        <v>1225048.075239</v>
+        <v>1429941.955596</v>
       </c>
       <c r="T124" t="n">
-        <v>1218864.058512</v>
+        <v>1412311.515923</v>
       </c>
       <c r="U124" t="n">
-        <v>1206329.637744</v>
+        <v>1388262.754241</v>
       </c>
       <c r="V124" t="n">
-        <v>1190130.522668</v>
+        <v>1360781.094377</v>
       </c>
     </row>
     <row r="125">
@@ -9874,58 +9874,58 @@
         </is>
       </c>
       <c r="E125" t="n">
-        <v>1275043.750695</v>
+        <v>973578.786989</v>
       </c>
       <c r="F125" t="n">
-        <v>1368643.28942</v>
+        <v>1036512.887472</v>
       </c>
       <c r="G125" t="n">
-        <v>1406767.814464</v>
+        <v>1048405.730492</v>
       </c>
       <c r="H125" t="n">
-        <v>1423628.070279</v>
+        <v>1053449.336668</v>
       </c>
       <c r="I125" t="n">
-        <v>1437457.16187</v>
+        <v>1064241.522168</v>
       </c>
       <c r="J125" t="n">
-        <v>1456404.918652</v>
+        <v>1084292.62393</v>
       </c>
       <c r="K125" t="n">
-        <v>1477687.793229</v>
+        <v>1109060.844847</v>
       </c>
       <c r="L125" t="n">
-        <v>1499736.105373</v>
+        <v>1135658.166907</v>
       </c>
       <c r="M125" t="n">
-        <v>1516086.248396</v>
+        <v>1158110.670436</v>
       </c>
       <c r="N125" t="n">
-        <v>1526724.01428</v>
+        <v>1175527.52361</v>
       </c>
       <c r="O125" t="n">
-        <v>1520854.43692</v>
+        <v>1179262.422725</v>
       </c>
       <c r="P125" t="n">
-        <v>1506903.135109</v>
+        <v>1175268.414031</v>
       </c>
       <c r="Q125" t="n">
-        <v>1485673.98003</v>
+        <v>1164786.287492</v>
       </c>
       <c r="R125" t="n">
-        <v>1455005.511274</v>
+        <v>1147106.754468</v>
       </c>
       <c r="S125" t="n">
-        <v>1416784.779074</v>
+        <v>1123035.497769</v>
       </c>
       <c r="T125" t="n">
-        <v>1373335.352457</v>
+        <v>1094402.187804</v>
       </c>
       <c r="U125" t="n">
-        <v>1326064.139247</v>
+        <v>1062381.981876</v>
       </c>
       <c r="V125" t="n">
-        <v>1277939.804454</v>
+        <v>1029425.682749</v>
       </c>
     </row>
     <row r="126">
@@ -14130,58 +14130,58 @@
         </is>
       </c>
       <c r="E181" t="n">
-        <v>4e-06</v>
+        <v>1e-06</v>
       </c>
       <c r="F181" t="n">
-        <v>4e-06</v>
+        <v>7e-06</v>
       </c>
       <c r="G181" t="n">
-        <v>-1e-06</v>
+        <v>-5e-06</v>
       </c>
       <c r="H181" t="n">
-        <v>-6e-06</v>
+        <v>2e-06</v>
       </c>
       <c r="I181" t="n">
-        <v>3e-06</v>
+        <v>5e-06</v>
       </c>
       <c r="J181" t="n">
-        <v>-4e-06</v>
+        <v>1e-06</v>
       </c>
       <c r="K181" t="n">
-        <v>6e-06</v>
+        <v>2e-06</v>
       </c>
       <c r="L181" t="n">
-        <v>4e-06</v>
+        <v>5e-06</v>
       </c>
       <c r="M181" t="n">
         <v>-5e-06</v>
       </c>
       <c r="N181" t="n">
-        <v>5e-06</v>
+        <v>4e-06</v>
       </c>
       <c r="O181" t="n">
+        <v>8e-06</v>
+      </c>
+      <c r="P181" t="n">
+        <v>1e-06</v>
+      </c>
+      <c r="Q181" t="n">
         <v>2e-06</v>
       </c>
-      <c r="P181" t="n">
+      <c r="R181" t="n">
+        <v>-3e-06</v>
+      </c>
+      <c r="S181" t="n">
+        <v>-3e-06</v>
+      </c>
+      <c r="T181" t="n">
         <v>3e-06</v>
       </c>
-      <c r="Q181" t="n">
-        <v>-0</v>
-      </c>
-      <c r="R181" t="n">
-        <v>-5e-06</v>
-      </c>
-      <c r="S181" t="n">
-        <v>4e-06</v>
-      </c>
-      <c r="T181" t="n">
-        <v>5e-06</v>
-      </c>
       <c r="U181" t="n">
-        <v>-4e-06</v>
+        <v>-8e-06</v>
       </c>
       <c r="V181" t="n">
-        <v>1e-06</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>